<commit_message>
Flexible Dólar: quitar marzo (mes de inicio abril) para que el folleto muestre solo mayo y junio
El fondo partió en abril, así que abril es el mes base (sin mes previo para comparar)
y no debe mostrar rentabilidad. Se blanquea el punto de marzo (col G) del template;
así abril queda como base y la tabla muestra solo mayo y junio.
</commit_message>
<xml_diff>
--- a/inputs/templates/TEMPLATE FONDO LIQUIDEZ FLEXIBLE DOLAR.xlsx
+++ b/inputs/templates/TEMPLATE FONDO LIQUIDEZ FLEXIBLE DOLAR.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW99"/>
+  <dimension ref="A1:AW19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,15 +463,7 @@
       <c r="B3" t="n">
         <v>26333.64</v>
       </c>
-      <c r="F3" s="1" t="n">
-        <v>46112</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F3" s="1" t="n"/>
       <c r="K3" t="n">
         <v>1460.0275</v>
       </c>
@@ -597,86 +589,6 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>